<commit_message>
#4 Fresh Deliverables Generated along with fresh Client BOM.
</commit_message>
<xml_diff>
--- a/Design-Files/GamingMouse-v1.1/BOM/Client_BOM_GamingMouse-v1.1.xlsx
+++ b/Design-Files/GamingMouse-v1.1/BOM/Client_BOM_GamingMouse-v1.1.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\austingunniers-gamingmouse\Design-Files\GamingMouse-v1.1\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LiberDB\Documents\GitHub\austingunniers-gamingmouse\Design-Files\GamingMouse-v1.1\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -14,12 +14,15 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$P$1:$R$70</definedName>
+  </definedNames>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="321">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="322">
   <si>
     <t>#</t>
   </si>
@@ -66,9 +69,6 @@
     <t>Resistor</t>
   </si>
   <si>
-    <t>Slide Switche</t>
-  </si>
-  <si>
     <t>Mouse Micro Switch</t>
   </si>
   <si>
@@ -249,9 +249,6 @@
     <t>R31</t>
   </si>
   <si>
-    <t>Slide Switch1</t>
-  </si>
-  <si>
     <t>SW1, SW2, SW3, SW6, SW7</t>
   </si>
   <si>
@@ -982,13 +979,22 @@
   </si>
   <si>
     <t>3.7v 200mah 401020 Lithium Polymer Li-po Rechargeable Battery For Toys Cars Bluetooth Speaker Bluetooth Headset Digital Products</t>
+  </si>
+  <si>
+    <t>AliExpress</t>
+  </si>
+  <si>
+    <t>Slide Switch</t>
+  </si>
+  <si>
+    <t>SW9</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1035,6 +1041,14 @@
       <strike/>
       <sz val="9"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1152,10 +1166,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1192,17 +1207,21 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1501,6 +1520,9 @@
     <col min="9" max="9" width="6.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="16.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="29.42578125" customWidth="1"/>
+    <col min="13" max="13" width="36" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="33.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="16.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1512,9 +1534,9 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1525,28 +1547,28 @@
         <v>1</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1559,22 +1581,22 @@
         <v>2</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J3" s="7">
         <v>1</v>
@@ -1591,22 +1613,22 @@
         <v>3</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="J4" s="9">
         <v>3</v>
@@ -1623,22 +1645,22 @@
         <v>3</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="J5" s="7">
         <v>2</v>
@@ -1655,22 +1677,22 @@
         <v>3</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="J6" s="9">
         <v>6</v>
@@ -1687,22 +1709,22 @@
         <v>3</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="J7" s="7">
         <v>1</v>
@@ -1719,22 +1741,22 @@
         <v>3</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="J8" s="9">
         <v>1</v>
@@ -1751,22 +1773,22 @@
         <v>3</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="J9" s="7">
         <v>1</v>
@@ -1783,22 +1805,22 @@
         <v>3</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="J10" s="9">
         <v>1</v>
@@ -1815,22 +1837,22 @@
         <v>3</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="J11" s="7">
         <v>1</v>
@@ -1847,22 +1869,22 @@
         <v>3</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="J12" s="9">
         <v>1</v>
@@ -1879,22 +1901,22 @@
         <v>3</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="J13" s="7">
         <v>1</v>
@@ -1911,22 +1933,22 @@
         <v>3</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="J14" s="9">
         <v>1</v>
@@ -1943,22 +1965,22 @@
         <v>3</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="J15" s="7">
         <v>4</v>
@@ -1975,22 +1997,22 @@
         <v>3</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="J16" s="9">
         <v>1</v>
@@ -2007,22 +2029,22 @@
         <v>3</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="J17" s="7">
         <v>1</v>
@@ -2039,22 +2061,22 @@
         <v>3</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="J18" s="9">
         <v>7</v>
@@ -2071,22 +2093,22 @@
         <v>3</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="J19" s="7">
         <v>1</v>
@@ -2103,22 +2125,22 @@
         <v>3</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="J20" s="9">
         <v>1</v>
@@ -2134,28 +2156,28 @@
       <c r="C21" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="D21" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="E21" s="16" t="s">
-        <v>108</v>
-      </c>
-      <c r="F21" s="15" t="s">
-        <v>159</v>
-      </c>
-      <c r="G21" s="16" t="s">
-        <v>207</v>
-      </c>
-      <c r="H21" s="15" t="s">
-        <v>253</v>
-      </c>
-      <c r="I21" s="16" t="s">
-        <v>292</v>
-      </c>
-      <c r="J21" s="15">
+      <c r="D21" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="E21" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="F21" s="14" t="s">
+        <v>157</v>
+      </c>
+      <c r="G21" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="H21" s="14" t="s">
+        <v>251</v>
+      </c>
+      <c r="I21" s="15" t="s">
+        <v>290</v>
+      </c>
+      <c r="J21" s="14">
         <v>2</v>
       </c>
-      <c r="K21" s="15"/>
+      <c r="K21" s="14"/>
     </row>
     <row r="22" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
@@ -2167,22 +2189,22 @@
         <v>3</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="J22" s="9">
         <v>1</v>
@@ -2199,22 +2221,22 @@
         <v>3</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="J23" s="7">
         <v>1</v>
@@ -2231,22 +2253,22 @@
         <v>3</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="J24" s="9">
         <v>1</v>
@@ -2263,22 +2285,22 @@
         <v>4</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J25" s="7">
         <v>1</v>
@@ -2295,22 +2317,22 @@
         <v>5</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="J26" s="9">
         <v>3</v>
@@ -2327,22 +2349,22 @@
         <v>6</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J27" s="7">
         <v>1</v>
@@ -2359,22 +2381,22 @@
         <v>7</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="I28" s="8" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J28" s="9">
         <v>1</v>
@@ -2391,18 +2413,18 @@
         <v>7</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="G29" s="8"/>
       <c r="H29" s="7"/>
       <c r="I29" s="8" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J29" s="7">
         <v>1</v>
@@ -2419,22 +2441,22 @@
         <v>8</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="J30" s="9">
         <v>1</v>
@@ -2451,22 +2473,22 @@
         <v>9</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="J31" s="7">
         <v>1</v>
@@ -2483,22 +2505,22 @@
         <v>9</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="J32" s="9">
         <v>1</v>
@@ -2515,22 +2537,22 @@
         <v>9</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J33" s="7">
         <v>1</v>
@@ -2547,22 +2569,22 @@
         <v>10</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="G34" s="10" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I34" s="8" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J34" s="9">
         <v>1</v>
@@ -2579,22 +2601,22 @@
         <v>10</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J35" s="7">
         <v>1</v>
@@ -2611,22 +2633,22 @@
         <v>10</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="G36" s="10" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I36" s="8" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J36" s="9">
         <v>1</v>
@@ -2643,22 +2665,22 @@
         <v>11</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="H37" s="7" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="I37" s="8" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J37" s="7">
         <v>1</v>
@@ -2675,20 +2697,20 @@
         <v>12</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="F38" s="7" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="G38" s="9" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="H38" s="9"/>
       <c r="I38" s="8" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J38" s="9">
         <v>4</v>
@@ -2705,22 +2727,22 @@
         <v>13</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="F39" s="7" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="H39" s="7" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="I39" s="8" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J39" s="7">
         <v>1</v>
@@ -2737,22 +2759,22 @@
         <v>13</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="G40" s="10" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="H40" s="9" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="I40" s="8" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J40" s="9">
         <v>1</v>
@@ -2769,22 +2791,22 @@
         <v>13</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F41" s="7" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="G41" s="8" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="H41" s="7" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="I41" s="8" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J41" s="7">
         <v>1</v>
@@ -2801,22 +2823,22 @@
         <v>14</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E42" s="10" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="G42" s="10" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="H42" s="9" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="I42" s="10" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="J42" s="9">
         <v>1</v>
@@ -2831,22 +2853,22 @@
       </c>
       <c r="C43" s="12"/>
       <c r="D43" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="G43" s="8" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="H43" s="7" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="I43" s="8" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="J43" s="7">
         <v>2</v>
@@ -2863,22 +2885,22 @@
         <v>14</v>
       </c>
       <c r="D44" s="9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E44" s="10" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="G44" s="10" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="H44" s="9" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="I44" s="10" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="J44" s="9">
         <v>1</v>
@@ -2895,22 +2917,22 @@
         <v>14</v>
       </c>
       <c r="D45" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="F45" s="7" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="G45" s="8" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="H45" s="7" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="I45" s="8" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="J45" s="7">
         <v>1</v>
@@ -2927,22 +2949,22 @@
         <v>14</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="G46" s="10" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="H46" s="9" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="I46" s="10" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="J46" s="9">
         <v>12</v>
@@ -2959,22 +2981,22 @@
         <v>14</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F47" s="7" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="H47" s="7" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="I47" s="8" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="J47" s="7">
         <v>1</v>
@@ -2991,22 +3013,22 @@
         <v>14</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E48" s="10" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="G48" s="10" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="H48" s="9" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="I48" s="10" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="J48" s="9">
         <v>5</v>
@@ -3023,22 +3045,22 @@
         <v>14</v>
       </c>
       <c r="D49" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="H49" s="7" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I49" s="8" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="J49" s="7">
         <v>1</v>
@@ -3055,22 +3077,22 @@
         <v>14</v>
       </c>
       <c r="D50" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E50" s="10" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F50" s="9" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="G50" s="10" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="H50" s="9" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="I50" s="10" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="J50" s="9">
         <v>2</v>
@@ -3087,22 +3109,22 @@
         <v>14</v>
       </c>
       <c r="D51" s="7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F51" s="7" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="G51" s="8" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="H51" s="7" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="I51" s="8" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="J51" s="7">
         <v>1</v>
@@ -3118,28 +3140,28 @@
       <c r="C52" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="D52" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="E52" s="16" t="s">
-        <v>137</v>
-      </c>
-      <c r="F52" s="15" t="s">
-        <v>176</v>
-      </c>
-      <c r="G52" s="16" t="s">
-        <v>232</v>
-      </c>
-      <c r="H52" s="15" t="s">
-        <v>249</v>
-      </c>
-      <c r="I52" s="16" t="s">
-        <v>292</v>
-      </c>
-      <c r="J52" s="15">
-        <v>1</v>
-      </c>
-      <c r="K52" s="15"/>
+      <c r="D52" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="E52" s="15" t="s">
+        <v>135</v>
+      </c>
+      <c r="F52" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="G52" s="15" t="s">
+        <v>230</v>
+      </c>
+      <c r="H52" s="14" t="s">
+        <v>247</v>
+      </c>
+      <c r="I52" s="15" t="s">
+        <v>290</v>
+      </c>
+      <c r="J52" s="14">
+        <v>1</v>
+      </c>
+      <c r="K52" s="14"/>
     </row>
     <row r="53" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="1"/>
@@ -3151,22 +3173,22 @@
         <v>14</v>
       </c>
       <c r="D53" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E53" s="8" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F53" s="7" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="G53" s="8" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="H53" s="7" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="I53" s="8" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="J53" s="7">
         <v>1</v>
@@ -3183,22 +3205,22 @@
         <v>14</v>
       </c>
       <c r="D54" s="9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E54" s="10" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="F54" s="9" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="G54" s="10" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="H54" s="9" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="I54" s="10" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="J54" s="9">
         <v>1</v>
@@ -3215,22 +3237,22 @@
         <v>14</v>
       </c>
       <c r="D55" s="7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E55" s="8" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F55" s="7" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="G55" s="8" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="H55" s="7" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="I55" s="8" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="J55" s="7">
         <v>1</v>
@@ -3247,22 +3269,22 @@
         <v>14</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E56" s="10" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="F56" s="9" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="G56" s="10" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="H56" s="9" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I56" s="10" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="J56" s="9">
         <v>1</v>
@@ -3276,25 +3298,25 @@
         <v>55</v>
       </c>
       <c r="C57" s="12" t="s">
-        <v>15</v>
+        <v>320</v>
       </c>
       <c r="D57" s="7" t="s">
-        <v>76</v>
+        <v>321</v>
       </c>
       <c r="E57" s="8" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="F57" s="9" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="G57" s="8" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="H57" s="7" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="I57" s="8" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J57" s="7">
         <v>1</v>
@@ -3308,25 +3330,25 @@
         <v>56</v>
       </c>
       <c r="C58" s="13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D58" s="9" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E58" s="10" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="F58" s="9" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="G58" s="10" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="H58" s="9" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="I58" s="8" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J58" s="9">
         <v>5</v>
@@ -3340,25 +3362,25 @@
         <v>57</v>
       </c>
       <c r="C59" s="12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D59" s="7" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E59" s="8" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="F59" s="9" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="G59" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="H59" s="7" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I59" s="8" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J59" s="7">
         <v>1</v>
@@ -3373,20 +3395,20 @@
       </c>
       <c r="C60" s="13"/>
       <c r="D60" s="9" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E60" s="10" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="F60" s="9" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="G60" s="10" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="H60" s="9"/>
       <c r="I60" s="8" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J60" s="9">
         <v>1</v>
@@ -3400,25 +3422,25 @@
         <v>59</v>
       </c>
       <c r="C61" s="12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D61" s="7" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E61" s="8" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F61" s="9" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="G61" s="8" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="H61" s="7" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="I61" s="8" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J61" s="7">
         <v>1</v>
@@ -3432,25 +3454,25 @@
         <v>60</v>
       </c>
       <c r="C62" s="13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D62" s="9" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E62" s="10" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="F62" s="9" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G62" s="10" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="H62" s="9" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I62" s="8" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J62" s="9">
         <v>2</v>
@@ -3464,25 +3486,25 @@
         <v>61</v>
       </c>
       <c r="C63" s="12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D63" s="7" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="E63" s="8" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F63" s="9" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="G63" s="8" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="H63" s="7" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="I63" s="8" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J63" s="7">
         <v>1</v>
@@ -3497,22 +3519,22 @@
       </c>
       <c r="C64" s="13"/>
       <c r="D64" s="9" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E64" s="10" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F64" s="9" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G64" s="10" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="H64" s="9" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="I64" s="8" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J64" s="9">
         <v>1</v>
@@ -3526,25 +3548,25 @@
         <v>63</v>
       </c>
       <c r="C65" s="12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D65" s="7" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="E65" s="8" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="F65" s="7" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="G65" s="8" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="H65" s="7" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="I65" s="8" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J65" s="7">
         <v>1</v>
@@ -3558,25 +3580,25 @@
         <v>64</v>
       </c>
       <c r="C66" s="13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D66" s="9" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E66" s="10" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F66" s="9" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G66" s="10" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="H66" s="9" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="I66" s="8" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J66" s="9">
         <v>1</v>
@@ -3590,25 +3612,25 @@
         <v>65</v>
       </c>
       <c r="C67" s="12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D67" s="7" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E67" s="8" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="F67" s="7" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="G67" s="8" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="H67" s="7" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="I67" s="8" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="J67" s="7">
         <v>1</v>
@@ -3622,25 +3644,25 @@
         <v>66</v>
       </c>
       <c r="C68" s="13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D68" s="9" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="E68" s="10" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="F68" s="9" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="G68" s="10" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="H68" s="9" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="I68" s="10" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="J68" s="9">
         <v>1</v>
@@ -3654,30 +3676,30 @@
         <v>67</v>
       </c>
       <c r="C69" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="D69" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="E69" s="16" t="s">
-        <v>155</v>
-      </c>
-      <c r="F69" s="15" t="s">
-        <v>188</v>
-      </c>
-      <c r="G69" s="16" t="s">
-        <v>244</v>
-      </c>
-      <c r="H69" s="15" t="s">
-        <v>277</v>
-      </c>
-      <c r="I69" s="16" t="s">
-        <v>292</v>
-      </c>
-      <c r="J69" s="15">
-        <v>1</v>
-      </c>
-      <c r="K69" s="15"/>
+        <v>19</v>
+      </c>
+      <c r="D69" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="E69" s="15" t="s">
+        <v>153</v>
+      </c>
+      <c r="F69" s="14" t="s">
+        <v>186</v>
+      </c>
+      <c r="G69" s="15" t="s">
+        <v>242</v>
+      </c>
+      <c r="H69" s="14" t="s">
+        <v>275</v>
+      </c>
+      <c r="I69" s="15" t="s">
+        <v>290</v>
+      </c>
+      <c r="J69" s="14">
+        <v>1</v>
+      </c>
+      <c r="K69" s="14"/>
     </row>
     <row r="70" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B70" s="11">
@@ -3685,36 +3707,41 @@
         <v>68</v>
       </c>
       <c r="C70" s="13" t="s">
+        <v>316</v>
+      </c>
+      <c r="D70" s="9" t="s">
+        <v>313</v>
+      </c>
+      <c r="E70" s="10" t="s">
         <v>318</v>
       </c>
-      <c r="D70" s="9" t="s">
-        <v>315</v>
-      </c>
-      <c r="E70" s="10" t="s">
-        <v>320</v>
-      </c>
       <c r="F70" s="9" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="G70" s="10" t="s">
+        <v>317</v>
+      </c>
+      <c r="H70" s="9" t="s">
+        <v>313</v>
+      </c>
+      <c r="I70" s="10" t="s">
+        <v>313</v>
+      </c>
+      <c r="J70" s="9">
+        <v>1</v>
+      </c>
+      <c r="K70" s="16" t="s">
         <v>319</v>
       </c>
-      <c r="H70" s="9" t="s">
-        <v>315</v>
-      </c>
-      <c r="I70" s="10" t="s">
-        <v>315</v>
-      </c>
-      <c r="J70" s="9">
-        <v>1</v>
-      </c>
-      <c r="K70" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="I1:K1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="K70" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
#4 PCB changes after review in #3
</commit_message>
<xml_diff>
--- a/Design-Files/GamingMouse-v1.1/BOM/Client_BOM_GamingMouse-v1.1.xlsx
+++ b/Design-Files/GamingMouse-v1.1/BOM/Client_BOM_GamingMouse-v1.1.xlsx
@@ -5,24 +5,24 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LiberDB\Documents\GitHub\austingunniers-gamingmouse\Design-Files\GamingMouse-v1.1\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MarsVirgo\Downloads\austingunniers-gamingmouse\austingunniers-gamingmouse-Development-v1.1\Design-Files\GamingMouse-v1.1\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7620"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$P$1:$R$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$P$1:$R$71</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="328">
   <si>
     <t>#</t>
   </si>
@@ -222,9 +222,6 @@
     <t>R7</t>
   </si>
   <si>
-    <t>R9, R10, R11, R27, R29</t>
-  </si>
-  <si>
     <t>R12</t>
   </si>
   <si>
@@ -988,6 +985,27 @@
   </si>
   <si>
     <t>SW9</t>
+  </si>
+  <si>
+    <t>R27, R29</t>
+  </si>
+  <si>
+    <t>R9, R10, R11</t>
+  </si>
+  <si>
+    <t>330R</t>
+  </si>
+  <si>
+    <t>CRCW0402330RFKEDC</t>
+  </si>
+  <si>
+    <t>SMD Chip Resistor, 330 Ohm, ± 1%, 63 mW, 0402 [1005 Metric], Thick Film, General Purpose</t>
+  </si>
+  <si>
+    <t>Res-0403</t>
+  </si>
+  <si>
+    <t>Encoder</t>
   </si>
 </sst>
 </file>
@@ -1507,14 +1525,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K70"/>
+  <dimension ref="A1:K71"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
     <col min="3" max="3" width="18.7109375" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="26.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.5703125" customWidth="1"/>
     <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="6.85546875" bestFit="1" customWidth="1"/>
@@ -1550,25 +1568,25 @@
         <v>20</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1584,19 +1602,19 @@
         <v>21</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="J3" s="7">
         <v>1</v>
@@ -1606,7 +1624,7 @@
     <row r="4" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
-        <f t="shared" ref="B4:B68" si="0">ROW(B4) - ROW($B$2)</f>
+        <f t="shared" ref="B4:B69" si="0">ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
       <c r="C4" s="12" t="s">
@@ -1616,19 +1634,19 @@
         <v>22</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="J4" s="9">
         <v>3</v>
@@ -1648,19 +1666,19 @@
         <v>23</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="J5" s="7">
         <v>2</v>
@@ -1680,19 +1698,19 @@
         <v>24</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="J6" s="9">
         <v>6</v>
@@ -1712,19 +1730,19 @@
         <v>25</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="J7" s="7">
         <v>1</v>
@@ -1744,19 +1762,19 @@
         <v>26</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="J8" s="9">
         <v>1</v>
@@ -1776,19 +1794,19 @@
         <v>27</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="J9" s="7">
         <v>1</v>
@@ -1808,19 +1826,19 @@
         <v>28</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="J10" s="9">
         <v>1</v>
@@ -1840,19 +1858,19 @@
         <v>29</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="J11" s="7">
         <v>1</v>
@@ -1872,19 +1890,19 @@
         <v>30</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="J12" s="9">
         <v>1</v>
@@ -1904,19 +1922,19 @@
         <v>31</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="J13" s="7">
         <v>1</v>
@@ -1936,19 +1954,19 @@
         <v>32</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="J14" s="9">
         <v>1</v>
@@ -1968,19 +1986,19 @@
         <v>33</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="J15" s="7">
         <v>4</v>
@@ -2000,19 +2018,19 @@
         <v>34</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="J16" s="9">
         <v>1</v>
@@ -2032,19 +2050,19 @@
         <v>35</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="J17" s="7">
         <v>1</v>
@@ -2064,19 +2082,19 @@
         <v>36</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="J18" s="9">
         <v>7</v>
@@ -2096,19 +2114,19 @@
         <v>37</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="J19" s="7">
         <v>1</v>
@@ -2128,19 +2146,19 @@
         <v>38</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="J20" s="9">
         <v>1</v>
@@ -2160,19 +2178,19 @@
         <v>39</v>
       </c>
       <c r="E21" s="15" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F21" s="14" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G21" s="15" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="H21" s="14" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="I21" s="15" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="J21" s="14">
         <v>2</v>
@@ -2192,19 +2210,19 @@
         <v>40</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="J22" s="9">
         <v>1</v>
@@ -2224,19 +2242,19 @@
         <v>41</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="J23" s="7">
         <v>1</v>
@@ -2256,19 +2274,19 @@
         <v>42</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="J24" s="9">
         <v>1</v>
@@ -2288,19 +2306,19 @@
         <v>43</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="J25" s="7">
         <v>1</v>
@@ -2320,19 +2338,19 @@
         <v>44</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="J26" s="9">
         <v>3</v>
@@ -2352,19 +2370,19 @@
         <v>45</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="J27" s="7">
         <v>1</v>
@@ -2384,19 +2402,19 @@
         <v>46</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="I28" s="8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="J28" s="9">
         <v>1</v>
@@ -2416,15 +2434,15 @@
         <v>47</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="G29" s="8"/>
       <c r="H29" s="7"/>
       <c r="I29" s="8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="J29" s="7">
         <v>1</v>
@@ -2444,19 +2462,19 @@
         <v>48</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="J30" s="9">
         <v>1</v>
@@ -2476,19 +2494,19 @@
         <v>49</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="J31" s="7">
         <v>1</v>
@@ -2508,19 +2526,19 @@
         <v>50</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="J32" s="9">
         <v>1</v>
@@ -2540,19 +2558,19 @@
         <v>51</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="J33" s="7">
         <v>1</v>
@@ -2572,19 +2590,19 @@
         <v>52</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="G34" s="10" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="I34" s="8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="J34" s="9">
         <v>1</v>
@@ -2604,19 +2622,19 @@
         <v>53</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="J35" s="7">
         <v>1</v>
@@ -2636,19 +2654,19 @@
         <v>54</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="G36" s="10" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="I36" s="8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="J36" s="9">
         <v>1</v>
@@ -2668,19 +2686,19 @@
         <v>55</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H37" s="7" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="I37" s="8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="J37" s="7">
         <v>1</v>
@@ -2700,17 +2718,17 @@
         <v>56</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F38" s="7" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="G38" s="9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H38" s="9"/>
       <c r="I38" s="8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="J38" s="9">
         <v>4</v>
@@ -2730,19 +2748,19 @@
         <v>57</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F39" s="7" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H39" s="7" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="I39" s="8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="J39" s="7">
         <v>1</v>
@@ -2762,19 +2780,19 @@
         <v>58</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="G40" s="10" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="H40" s="9" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="I40" s="8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="J40" s="9">
         <v>1</v>
@@ -2794,19 +2812,19 @@
         <v>59</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F41" s="7" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G41" s="8" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H41" s="7" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="I41" s="8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="J41" s="7">
         <v>1</v>
@@ -2826,19 +2844,19 @@
         <v>60</v>
       </c>
       <c r="E42" s="10" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G42" s="10" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="H42" s="9" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="I42" s="10" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="J42" s="9">
         <v>1</v>
@@ -2856,19 +2874,19 @@
         <v>61</v>
       </c>
       <c r="E43" s="8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G43" s="8" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="H43" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I43" s="8" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="J43" s="7">
         <v>2</v>
@@ -2888,19 +2906,19 @@
         <v>62</v>
       </c>
       <c r="E44" s="10" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="G44" s="10" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H44" s="9" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I44" s="10" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="J44" s="9">
         <v>1</v>
@@ -2920,19 +2938,19 @@
         <v>63</v>
       </c>
       <c r="E45" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F45" s="7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="G45" s="8" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="H45" s="7" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="I45" s="8" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="J45" s="7">
         <v>1</v>
@@ -2952,19 +2970,19 @@
         <v>64</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G46" s="10" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="H46" s="9" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I46" s="10" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="J46" s="9">
         <v>12</v>
@@ -2984,26 +3002,26 @@
         <v>65</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F47" s="7" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H47" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I47" s="8" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J47" s="7">
         <v>1</v>
       </c>
       <c r="K47" s="7"/>
     </row>
-    <row r="48" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1"/>
       <c r="B48" s="11">
         <f t="shared" si="0"/>
@@ -3013,25 +3031,25 @@
         <v>14</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="E48" s="10" t="s">
-        <v>133</v>
+        <v>322</v>
+      </c>
+      <c r="E48" s="8" t="s">
+        <v>325</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>174</v>
-      </c>
-      <c r="G48" s="10" t="s">
-        <v>228</v>
-      </c>
-      <c r="H48" s="9" t="s">
-        <v>247</v>
+        <v>173</v>
+      </c>
+      <c r="G48" s="8" t="s">
+        <v>324</v>
+      </c>
+      <c r="H48" s="7" t="s">
+        <v>251</v>
       </c>
       <c r="I48" s="10" t="s">
-        <v>302</v>
+        <v>323</v>
       </c>
       <c r="J48" s="9">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K48" s="9"/>
     </row>
@@ -3045,22 +3063,22 @@
         <v>14</v>
       </c>
       <c r="D49" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="H49" s="7" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="I49" s="8" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="J49" s="7">
         <v>1</v>
@@ -3077,22 +3095,22 @@
         <v>14</v>
       </c>
       <c r="D50" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E50" s="10" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F50" s="9" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G50" s="10" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="H50" s="9" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I50" s="10" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="J50" s="9">
         <v>2</v>
@@ -3109,22 +3127,22 @@
         <v>14</v>
       </c>
       <c r="D51" s="7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E51" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F51" s="7" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G51" s="8" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H51" s="7" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="I51" s="8" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="J51" s="7">
         <v>1</v>
@@ -3141,22 +3159,22 @@
         <v>14</v>
       </c>
       <c r="D52" s="14" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E52" s="15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F52" s="14" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G52" s="15" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="H52" s="14" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I52" s="15" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="J52" s="14">
         <v>1</v>
@@ -3173,22 +3191,22 @@
         <v>14</v>
       </c>
       <c r="D53" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E53" s="8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F53" s="7" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G53" s="8" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="H53" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I53" s="8" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="J53" s="7">
         <v>1</v>
@@ -3198,540 +3216,575 @@
     <row r="54" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="1"/>
       <c r="B54" s="11">
-        <f t="shared" si="0"/>
         <v>52</v>
       </c>
-      <c r="C54" s="13" t="s">
+      <c r="C54" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="D54" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="E54" s="10" t="s">
-        <v>138</v>
-      </c>
-      <c r="F54" s="9" t="s">
-        <v>174</v>
+      <c r="D54" s="7" t="s">
+        <v>321</v>
+      </c>
+      <c r="E54" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="F54" s="7" t="s">
+        <v>326</v>
       </c>
       <c r="G54" s="10" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="H54" s="9" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="I54" s="10" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="J54" s="9">
-        <v>1</v>
-      </c>
-      <c r="K54" s="9"/>
+        <v>2</v>
+      </c>
+      <c r="K54" s="7"/>
     </row>
     <row r="55" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="1"/>
       <c r="B55" s="11">
-        <f>ROW(B55) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>53</v>
       </c>
-      <c r="C55" s="12" t="s">
+      <c r="C55" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="D55" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="E55" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="F55" s="7" t="s">
-        <v>174</v>
-      </c>
-      <c r="G55" s="8" t="s">
-        <v>234</v>
-      </c>
-      <c r="H55" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="I55" s="8" t="s">
-        <v>307</v>
-      </c>
-      <c r="J55" s="7">
-        <v>1</v>
-      </c>
-      <c r="K55" s="7"/>
+      <c r="D55" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="E55" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="F55" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="G55" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="H55" s="9" t="s">
+        <v>246</v>
+      </c>
+      <c r="I55" s="10" t="s">
+        <v>305</v>
+      </c>
+      <c r="J55" s="9">
+        <v>1</v>
+      </c>
+      <c r="K55" s="9"/>
     </row>
     <row r="56" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1"/>
       <c r="B56" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B56) - ROW($B$2)</f>
         <v>54</v>
       </c>
-      <c r="C56" s="13" t="s">
+      <c r="C56" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="D56" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="E56" s="10" t="s">
-        <v>140</v>
-      </c>
-      <c r="F56" s="9" t="s">
-        <v>174</v>
-      </c>
-      <c r="G56" s="10" t="s">
-        <v>235</v>
-      </c>
-      <c r="H56" s="9" t="s">
-        <v>263</v>
-      </c>
-      <c r="I56" s="10" t="s">
-        <v>308</v>
-      </c>
-      <c r="J56" s="9">
-        <v>1</v>
-      </c>
-      <c r="K56" s="9"/>
+      <c r="D56" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="E56" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="F56" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="G56" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="H56" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="I56" s="8" t="s">
+        <v>306</v>
+      </c>
+      <c r="J56" s="7">
+        <v>1</v>
+      </c>
+      <c r="K56" s="7"/>
     </row>
     <row r="57" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1"/>
       <c r="B57" s="11">
-        <f>ROW(B57) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>55</v>
       </c>
-      <c r="C57" s="12" t="s">
-        <v>320</v>
-      </c>
-      <c r="D57" s="7" t="s">
-        <v>321</v>
-      </c>
-      <c r="E57" s="8" t="s">
-        <v>141</v>
+      <c r="C57" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D57" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="E57" s="10" t="s">
+        <v>139</v>
       </c>
       <c r="F57" s="9" t="s">
-        <v>314</v>
-      </c>
-      <c r="G57" s="8" t="s">
-        <v>175</v>
-      </c>
-      <c r="H57" s="7" t="s">
-        <v>265</v>
-      </c>
-      <c r="I57" s="8" t="s">
-        <v>313</v>
-      </c>
-      <c r="J57" s="7">
-        <v>1</v>
-      </c>
-      <c r="K57" s="7"/>
-    </row>
-    <row r="58" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>173</v>
+      </c>
+      <c r="G57" s="10" t="s">
+        <v>234</v>
+      </c>
+      <c r="H57" s="9" t="s">
+        <v>262</v>
+      </c>
+      <c r="I57" s="10" t="s">
+        <v>307</v>
+      </c>
+      <c r="J57" s="9">
+        <v>1</v>
+      </c>
+      <c r="K57" s="9"/>
+    </row>
+    <row r="58" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="1"/>
       <c r="B58" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B58) - ROW($B$2)</f>
         <v>56</v>
       </c>
-      <c r="C58" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="D58" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="E58" s="10" t="s">
-        <v>142</v>
+      <c r="C58" s="12" t="s">
+        <v>319</v>
+      </c>
+      <c r="D58" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="E58" s="8" t="s">
+        <v>140</v>
       </c>
       <c r="F58" s="9" t="s">
-        <v>314</v>
-      </c>
-      <c r="G58" s="10" t="s">
-        <v>176</v>
-      </c>
-      <c r="H58" s="9" t="s">
-        <v>266</v>
+        <v>313</v>
+      </c>
+      <c r="G58" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="H58" s="7" t="s">
+        <v>264</v>
       </c>
       <c r="I58" s="8" t="s">
-        <v>313</v>
-      </c>
-      <c r="J58" s="9">
-        <v>5</v>
-      </c>
-      <c r="K58" s="9"/>
-    </row>
-    <row r="59" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>312</v>
+      </c>
+      <c r="J58" s="7">
+        <v>1</v>
+      </c>
+      <c r="K58" s="7"/>
+    </row>
+    <row r="59" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="1"/>
       <c r="B59" s="11">
-        <f>ROW(B59) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>57</v>
       </c>
-      <c r="C59" s="12" t="s">
-        <v>16</v>
-      </c>
-      <c r="D59" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="E59" s="8" t="s">
-        <v>143</v>
+      <c r="C59" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D59" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="E59" s="10" t="s">
+        <v>141</v>
       </c>
       <c r="F59" s="9" t="s">
-        <v>314</v>
-      </c>
-      <c r="G59" s="8" t="s">
-        <v>177</v>
-      </c>
-      <c r="H59" s="7" t="s">
-        <v>267</v>
+        <v>313</v>
+      </c>
+      <c r="G59" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="H59" s="9" t="s">
+        <v>265</v>
       </c>
       <c r="I59" s="8" t="s">
-        <v>313</v>
-      </c>
-      <c r="J59" s="7">
-        <v>1</v>
-      </c>
-      <c r="K59" s="7"/>
+        <v>312</v>
+      </c>
+      <c r="J59" s="9">
+        <v>5</v>
+      </c>
+      <c r="K59" s="9"/>
     </row>
     <row r="60" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="1"/>
       <c r="B60" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B60) - ROW($B$2)</f>
         <v>58</v>
       </c>
-      <c r="C60" s="13"/>
-      <c r="D60" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="E60" s="10" t="s">
-        <v>144</v>
+      <c r="C60" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D60" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E60" s="8" t="s">
+        <v>142</v>
       </c>
       <c r="F60" s="9" t="s">
-        <v>314</v>
-      </c>
-      <c r="G60" s="10" t="s">
-        <v>178</v>
-      </c>
-      <c r="H60" s="9"/>
+        <v>313</v>
+      </c>
+      <c r="G60" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="H60" s="7" t="s">
+        <v>266</v>
+      </c>
       <c r="I60" s="8" t="s">
-        <v>313</v>
-      </c>
-      <c r="J60" s="9">
-        <v>1</v>
-      </c>
-      <c r="K60" s="9"/>
+        <v>312</v>
+      </c>
+      <c r="J60" s="7">
+        <v>1</v>
+      </c>
+      <c r="K60" s="7"/>
     </row>
     <row r="61" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="1"/>
       <c r="B61" s="11">
-        <f>ROW(B61) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>59</v>
       </c>
-      <c r="C61" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="D61" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="E61" s="8" t="s">
-        <v>145</v>
+      <c r="C61" s="13" t="s">
+        <v>327</v>
+      </c>
+      <c r="D61" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="E61" s="10" t="s">
+        <v>143</v>
       </c>
       <c r="F61" s="9" t="s">
-        <v>314</v>
-      </c>
-      <c r="G61" s="8" t="s">
-        <v>179</v>
-      </c>
-      <c r="H61" s="7" t="s">
-        <v>268</v>
-      </c>
+        <v>313</v>
+      </c>
+      <c r="G61" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="H61" s="9"/>
       <c r="I61" s="8" t="s">
-        <v>313</v>
-      </c>
-      <c r="J61" s="7">
-        <v>1</v>
-      </c>
-      <c r="K61" s="7"/>
+        <v>312</v>
+      </c>
+      <c r="J61" s="9">
+        <v>1</v>
+      </c>
+      <c r="K61" s="9"/>
     </row>
     <row r="62" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="1"/>
       <c r="B62" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B62) - ROW($B$2)</f>
         <v>60</v>
       </c>
-      <c r="C62" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="D62" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="E62" s="10" t="s">
-        <v>146</v>
+      <c r="C62" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D62" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="E62" s="8" t="s">
+        <v>144</v>
       </c>
       <c r="F62" s="9" t="s">
-        <v>180</v>
-      </c>
-      <c r="G62" s="10" t="s">
-        <v>236</v>
-      </c>
-      <c r="H62" s="9" t="s">
-        <v>269</v>
+        <v>313</v>
+      </c>
+      <c r="G62" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="H62" s="7" t="s">
+        <v>267</v>
       </c>
       <c r="I62" s="8" t="s">
-        <v>313</v>
-      </c>
-      <c r="J62" s="9">
-        <v>2</v>
-      </c>
-      <c r="K62" s="9"/>
-    </row>
-    <row r="63" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>312</v>
+      </c>
+      <c r="J62" s="7">
+        <v>1</v>
+      </c>
+      <c r="K62" s="7"/>
+    </row>
+    <row r="63" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="1"/>
       <c r="B63" s="11">
-        <f>ROW(B63) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>61</v>
       </c>
-      <c r="C63" s="12" t="s">
+      <c r="C63" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="D63" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="E63" s="8" t="s">
-        <v>147</v>
+      <c r="D63" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="E63" s="10" t="s">
+        <v>145</v>
       </c>
       <c r="F63" s="9" t="s">
-        <v>314</v>
-      </c>
-      <c r="G63" s="8" t="s">
-        <v>181</v>
-      </c>
-      <c r="H63" s="7" t="s">
-        <v>270</v>
+        <v>179</v>
+      </c>
+      <c r="G63" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="H63" s="9" t="s">
+        <v>268</v>
       </c>
       <c r="I63" s="8" t="s">
-        <v>313</v>
-      </c>
-      <c r="J63" s="7">
-        <v>1</v>
-      </c>
-      <c r="K63" s="7"/>
-    </row>
-    <row r="64" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>312</v>
+      </c>
+      <c r="J63" s="9">
+        <v>2</v>
+      </c>
+      <c r="K63" s="9"/>
+    </row>
+    <row r="64" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A64" s="1"/>
       <c r="B64" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B64) - ROW($B$2)</f>
         <v>62</v>
       </c>
-      <c r="C64" s="13"/>
-      <c r="D64" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="E64" s="10" t="s">
-        <v>148</v>
+      <c r="C64" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D64" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E64" s="8" t="s">
+        <v>146</v>
       </c>
       <c r="F64" s="9" t="s">
-        <v>182</v>
-      </c>
-      <c r="G64" s="10" t="s">
-        <v>237</v>
-      </c>
-      <c r="H64" s="9" t="s">
+        <v>313</v>
+      </c>
+      <c r="G64" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="H64" s="7" t="s">
         <v>269</v>
       </c>
       <c r="I64" s="8" t="s">
-        <v>313</v>
-      </c>
-      <c r="J64" s="9">
-        <v>1</v>
-      </c>
-      <c r="K64" s="9"/>
-    </row>
-    <row r="65" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>312</v>
+      </c>
+      <c r="J64" s="7">
+        <v>1</v>
+      </c>
+      <c r="K64" s="7"/>
+    </row>
+    <row r="65" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="1"/>
       <c r="B65" s="11">
-        <f>ROW(B65) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>63</v>
       </c>
       <c r="C65" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="D65" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="E65" s="8" t="s">
-        <v>149</v>
-      </c>
-      <c r="F65" s="7" t="s">
-        <v>183</v>
-      </c>
-      <c r="G65" s="8" t="s">
-        <v>238</v>
-      </c>
-      <c r="H65" s="7" t="s">
-        <v>271</v>
+      <c r="D65" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="E65" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="F65" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="G65" s="10" t="s">
+        <v>236</v>
+      </c>
+      <c r="H65" s="9" t="s">
+        <v>268</v>
       </c>
       <c r="I65" s="8" t="s">
-        <v>313</v>
-      </c>
-      <c r="J65" s="7">
-        <v>1</v>
-      </c>
-      <c r="K65" s="7"/>
-    </row>
-    <row r="66" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>312</v>
+      </c>
+      <c r="J65" s="9">
+        <v>1</v>
+      </c>
+      <c r="K65" s="9"/>
+    </row>
+    <row r="66" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="1"/>
       <c r="B66" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B66) - ROW($B$2)</f>
         <v>64</v>
       </c>
-      <c r="C66" s="13" t="s">
+      <c r="C66" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="D66" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="E66" s="10" t="s">
-        <v>150</v>
-      </c>
-      <c r="F66" s="9" t="s">
-        <v>180</v>
-      </c>
-      <c r="G66" s="10" t="s">
-        <v>239</v>
-      </c>
-      <c r="H66" s="9" t="s">
-        <v>272</v>
+      <c r="D66" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="E66" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="F66" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="G66" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="H66" s="7" t="s">
+        <v>270</v>
       </c>
       <c r="I66" s="8" t="s">
-        <v>313</v>
-      </c>
-      <c r="J66" s="9">
-        <v>1</v>
-      </c>
-      <c r="K66" s="9"/>
+        <v>312</v>
+      </c>
+      <c r="J66" s="7">
+        <v>1</v>
+      </c>
+      <c r="K66" s="7"/>
     </row>
     <row r="67" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="1"/>
       <c r="B67" s="11">
-        <f>ROW(B67) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>65</v>
       </c>
-      <c r="C67" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="D67" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="E67" s="8" t="s">
-        <v>151</v>
-      </c>
-      <c r="F67" s="7" t="s">
-        <v>184</v>
-      </c>
-      <c r="G67" s="8" t="s">
-        <v>240</v>
-      </c>
-      <c r="H67" s="7" t="s">
-        <v>273</v>
+      <c r="C67" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D67" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="E67" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="F67" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="G67" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="H67" s="9" t="s">
+        <v>271</v>
       </c>
       <c r="I67" s="8" t="s">
-        <v>309</v>
-      </c>
-      <c r="J67" s="7">
-        <v>1</v>
-      </c>
-      <c r="K67" s="7"/>
+        <v>312</v>
+      </c>
+      <c r="J67" s="9">
+        <v>1</v>
+      </c>
+      <c r="K67" s="9"/>
     </row>
     <row r="68" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A68" s="1"/>
       <c r="B68" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B68) - ROW($B$2)</f>
         <v>66</v>
       </c>
-      <c r="C68" s="13" t="s">
+      <c r="C68" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="D68" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="E68" s="10" t="s">
-        <v>152</v>
-      </c>
-      <c r="F68" s="9" t="s">
-        <v>185</v>
-      </c>
-      <c r="G68" s="10" t="s">
-        <v>241</v>
-      </c>
-      <c r="H68" s="9" t="s">
-        <v>274</v>
-      </c>
-      <c r="I68" s="10" t="s">
-        <v>310</v>
-      </c>
-      <c r="J68" s="9">
-        <v>1</v>
-      </c>
-      <c r="K68" s="9"/>
-    </row>
-    <row r="69" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D68" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="E68" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="F68" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="G68" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="H68" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="I68" s="8" t="s">
+        <v>308</v>
+      </c>
+      <c r="J68" s="7">
+        <v>1</v>
+      </c>
+      <c r="K68" s="7"/>
+    </row>
+    <row r="69" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="1"/>
       <c r="B69" s="11">
-        <f>ROW(B69) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>67</v>
       </c>
       <c r="C69" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="D69" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="E69" s="15" t="s">
-        <v>153</v>
-      </c>
-      <c r="F69" s="14" t="s">
-        <v>186</v>
-      </c>
-      <c r="G69" s="15" t="s">
-        <v>242</v>
-      </c>
-      <c r="H69" s="14" t="s">
-        <v>275</v>
-      </c>
-      <c r="I69" s="15" t="s">
-        <v>290</v>
-      </c>
-      <c r="J69" s="14">
-        <v>1</v>
-      </c>
-      <c r="K69" s="14"/>
-    </row>
-    <row r="70" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D69" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="E69" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="F69" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="G69" s="10" t="s">
+        <v>240</v>
+      </c>
+      <c r="H69" s="9" t="s">
+        <v>273</v>
+      </c>
+      <c r="I69" s="10" t="s">
+        <v>309</v>
+      </c>
+      <c r="J69" s="9">
+        <v>1</v>
+      </c>
+      <c r="K69" s="9"/>
+    </row>
+    <row r="70" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="1"/>
       <c r="B70" s="11">
         <f>ROW(B70) - ROW($B$2)</f>
         <v>68</v>
       </c>
       <c r="C70" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D70" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="E70" s="15" t="s">
+        <v>152</v>
+      </c>
+      <c r="F70" s="14" t="s">
+        <v>185</v>
+      </c>
+      <c r="G70" s="15" t="s">
+        <v>241</v>
+      </c>
+      <c r="H70" s="14" t="s">
+        <v>274</v>
+      </c>
+      <c r="I70" s="15" t="s">
+        <v>289</v>
+      </c>
+      <c r="J70" s="14">
+        <v>1</v>
+      </c>
+      <c r="K70" s="14"/>
+    </row>
+    <row r="71" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B71" s="11">
+        <f>ROW(B71) - ROW($B$2)</f>
+        <v>69</v>
+      </c>
+      <c r="C71" s="13" t="s">
+        <v>315</v>
+      </c>
+      <c r="D71" s="9" t="s">
+        <v>312</v>
+      </c>
+      <c r="E71" s="10" t="s">
+        <v>317</v>
+      </c>
+      <c r="F71" s="9" t="s">
+        <v>312</v>
+      </c>
+      <c r="G71" s="10" t="s">
         <v>316</v>
       </c>
-      <c r="D70" s="9" t="s">
-        <v>313</v>
-      </c>
-      <c r="E70" s="10" t="s">
+      <c r="H71" s="9" t="s">
+        <v>312</v>
+      </c>
+      <c r="I71" s="10" t="s">
+        <v>312</v>
+      </c>
+      <c r="J71" s="9">
+        <v>1</v>
+      </c>
+      <c r="K71" s="16" t="s">
         <v>318</v>
-      </c>
-      <c r="F70" s="9" t="s">
-        <v>313</v>
-      </c>
-      <c r="G70" s="10" t="s">
-        <v>317</v>
-      </c>
-      <c r="H70" s="9" t="s">
-        <v>313</v>
-      </c>
-      <c r="I70" s="10" t="s">
-        <v>313</v>
-      </c>
-      <c r="J70" s="9">
-        <v>1</v>
-      </c>
-      <c r="K70" s="16" t="s">
-        <v>319</v>
       </c>
     </row>
   </sheetData>
@@ -3739,7 +3792,7 @@
     <mergeCell ref="I1:K1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="K70" r:id="rId1"/>
+    <hyperlink ref="K71" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>

</xml_diff>